<commit_message>
Site updated: 2025-03-24 21:56:32
</commit_message>
<xml_diff>
--- a/Ladon/wiki.xlsx
+++ b/Ladon/wiki.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19095" windowHeight="8865" activeTab="5"/>
+    <workbookView windowWidth="19095" windowHeight="8865" firstSheet="3" activeTab="8"/>
   </bookViews>
   <sheets>
     <sheet name="信息收集(远程)" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="680">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="691">
   <si>
     <t>Ladon模块</t>
   </si>
@@ -424,6 +424,9 @@
     <t>多种方式查找真实IP</t>
   </si>
   <si>
+    <t>注：本表格仅限EXE内置功能，不包含外置POC或专用EXP</t>
+  </si>
+  <si>
     <t>MS17010</t>
   </si>
   <si>
@@ -437,6 +440,12 @@
   </si>
   <si>
     <t>CVE-2020-0796 SMBGhost</t>
+  </si>
+  <si>
+    <t>CVE-2024-55591</t>
+  </si>
+  <si>
+    <t>FortiGate防火墙 未授权RCE漏洞检测</t>
   </si>
   <si>
     <t>CVE-2024-47176</t>
@@ -1145,6 +1154,15 @@
 slui</t>
   </si>
   <si>
+    <t>RunTrustedInstaller</t>
+  </si>
+  <si>
+    <t>TrustedInstaller权限执行命令</t>
+  </si>
+  <si>
+    <t>RunTrustedInstaller RunTI</t>
+  </si>
+  <si>
     <t>RunSystem</t>
   </si>
   <si>
@@ -1368,6 +1386,21 @@
   </si>
   <si>
     <t>邮服 Exchange 密码爆破(.net &gt;= 4.0)</t>
+  </si>
+  <si>
+    <t>FortiGateScan</t>
+  </si>
+  <si>
+    <t>FortiGate 密码爆破 默认只允许3次</t>
+  </si>
+  <si>
+    <t>FortiGateScan FortiScan</t>
+  </si>
+  <si>
+    <t>FortiVpnScan</t>
+  </si>
+  <si>
+    <t>Forti Vpn 密码爆破 默认只允许3次</t>
   </si>
   <si>
     <t>WeblogicScan</t>
@@ -1801,7 +1834,7 @@
     <t>放行指定TCP端口</t>
   </si>
   <si>
-    <t>OpenTcp OpenTcpPort</t>
+    <t>OpenTcp TcpOpen</t>
   </si>
   <si>
     <t>DisableService</t>
@@ -1825,7 +1858,7 @@
     <t>放行指定UDP端口</t>
   </si>
   <si>
-    <t>OpenUdp OpenUdpPort</t>
+    <t>OpenUdp UdpOpen</t>
   </si>
   <si>
     <t>CloseTcp</t>
@@ -1834,7 +1867,7 @@
     <t>关闭指定TCP端口</t>
   </si>
   <si>
-    <t>CloseTcp CloseTcpPort</t>
+    <t>CloseTcp TcpClose</t>
   </si>
   <si>
     <t>CloseUdp</t>
@@ -1843,7 +1876,7 @@
     <t>关闭指定UDP端口</t>
   </si>
   <si>
-    <t>CloseUdp CloseUdpPort</t>
+    <t>CloseUdp UdpClose</t>
   </si>
   <si>
     <t>CloseSMB</t>
@@ -2131,7 +2164,7 @@
     <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="24">
+  <fonts count="27">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2155,6 +2188,20 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="20"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="20"/>
+      <color rgb="FFFF0000"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="宋体"/>
@@ -2164,6 +2211,13 @@
     <font>
       <sz val="12"/>
       <color theme="1" tint="0.5"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="20"/>
+      <color theme="1"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -2627,10 +2681,10 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="23" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -2639,137 +2693,137 @@
     <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="14" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="14" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="14" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -2779,11 +2833,20 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2794,10 +2857,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -2807,6 +2867,9 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -3126,13 +3189,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr/>
-  <dimension ref="A1:E54"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="4"/>
+  <dimension ref="A1:XFD58"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="15.125" customWidth="1"/>
     <col min="2" max="2" width="4.875" customWidth="1"/>
     <col min="3" max="3" width="35.75" customWidth="1"/>
-    <col min="4" max="4" width="19.375" style="10" customWidth="1"/>
+    <col min="4" max="4" width="19.375" style="12" customWidth="1"/>
     <col min="5" max="5" width="43.375" customWidth="1"/>
   </cols>
   <sheetData>
@@ -3143,7 +3206,7 @@
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="4" t="s">
         <v>2</v>
       </c>
       <c r="E1" s="1" t="s">
@@ -3157,7 +3220,7 @@
       <c r="C3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="11"/>
+      <c r="D3" s="13"/>
       <c r="E3" s="2" t="s">
         <v>6</v>
       </c>
@@ -3169,7 +3232,7 @@
       <c r="C4" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="11"/>
+      <c r="D4" s="13"/>
       <c r="E4" s="2" t="s">
         <v>9</v>
       </c>
@@ -3181,7 +3244,7 @@
       <c r="C5" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="11"/>
+      <c r="D5" s="13"/>
       <c r="E5" s="2" t="s">
         <v>12</v>
       </c>
@@ -3193,7 +3256,7 @@
       <c r="C6" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="11"/>
+      <c r="D6" s="13"/>
     </row>
     <row r="7" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A7" s="2" t="s">
@@ -3202,24 +3265,24 @@
       <c r="C7" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="11">
+      <c r="D7" s="13">
         <v>135</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="8" s="12" customFormat="1" ht="14.25" spans="1:5">
-      <c r="A8" s="12" t="s">
+    <row r="8" s="14" customFormat="1" ht="14.25" spans="1:5">
+      <c r="A8" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="C8" s="12" t="s">
+      <c r="C8" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="D8" s="13">
+      <c r="D8" s="16">
         <v>53</v>
       </c>
-      <c r="E8" s="12" t="s">
+      <c r="E8" s="14" t="s">
         <v>20</v>
       </c>
     </row>
@@ -3230,7 +3293,7 @@
       <c r="C9" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="D9" s="11" t="s">
+      <c r="D9" s="13" t="s">
         <v>23</v>
       </c>
       <c r="E9" s="2" t="s">
@@ -3244,7 +3307,7 @@
       <c r="C10" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D10" s="11" t="s">
+      <c r="D10" s="13" t="s">
         <v>27</v>
       </c>
       <c r="E10" s="2" t="s">
@@ -3258,7 +3321,7 @@
       <c r="C11" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="D11" s="11" t="s">
+      <c r="D11" s="13" t="s">
         <v>31</v>
       </c>
       <c r="E11" s="2" t="s">
@@ -3272,7 +3335,7 @@
       <c r="C12" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="D12" s="11" t="s">
+      <c r="D12" s="13" t="s">
         <v>35</v>
       </c>
     </row>
@@ -3283,7 +3346,7 @@
       <c r="C13" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="D13" s="11" t="s">
+      <c r="D13" s="13" t="s">
         <v>35</v>
       </c>
       <c r="E13" s="2" t="s">
@@ -3297,7 +3360,7 @@
       <c r="C14" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="D14" s="11" t="s">
+      <c r="D14" s="13" t="s">
         <v>41</v>
       </c>
     </row>
@@ -3308,7 +3371,7 @@
       <c r="C15" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="D15" s="11" t="s">
+      <c r="D15" s="13" t="s">
         <v>35</v>
       </c>
       <c r="E15" s="2" t="s">
@@ -3322,7 +3385,7 @@
       <c r="C16" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="D16" s="11">
+      <c r="D16" s="13">
         <v>139</v>
       </c>
     </row>
@@ -3333,12 +3396,12 @@
       <c r="C17" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="D17" s="11" t="s">
+      <c r="D17" s="13" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="18" s="2" customFormat="1" ht="14.25" spans="4:4">
-      <c r="D18" s="11"/>
+      <c r="D18" s="13"/>
     </row>
     <row r="19" s="2" customFormat="1" ht="14.25" spans="1:4">
       <c r="A19" s="2" t="s">
@@ -3347,7 +3410,7 @@
       <c r="C19" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="D19" s="11">
+      <c r="D19" s="13">
         <v>135</v>
       </c>
     </row>
@@ -3358,7 +3421,7 @@
       <c r="C20" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="D20" s="11">
+      <c r="D20" s="13">
         <v>445</v>
       </c>
     </row>
@@ -3369,7 +3432,7 @@
       <c r="C21" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="D21" s="11" t="s">
+      <c r="D21" s="13" t="s">
         <v>56</v>
       </c>
     </row>
@@ -3380,7 +3443,7 @@
       <c r="C22" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="D22" s="11">
+      <c r="D22" s="13">
         <v>1433</v>
       </c>
     </row>
@@ -3391,7 +3454,7 @@
       <c r="C23" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="D23" s="11">
+      <c r="D23" s="13">
         <v>3389</v>
       </c>
     </row>
@@ -3402,7 +3465,7 @@
       <c r="C24" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="D24" s="11" t="s">
+      <c r="D24" s="13" t="s">
         <v>35</v>
       </c>
     </row>
@@ -3413,7 +3476,7 @@
       <c r="C25" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="D25" s="11" t="s">
+      <c r="D25" s="13" t="s">
         <v>65</v>
       </c>
     </row>
@@ -3424,7 +3487,7 @@
       <c r="C26" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="D26" s="11">
+      <c r="D26" s="13">
         <v>137</v>
       </c>
     </row>
@@ -3435,7 +3498,7 @@
       <c r="C27" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="D27" s="11" t="s">
+      <c r="D27" s="13" t="s">
         <v>35</v>
       </c>
       <c r="E27" s="2" t="s">
@@ -3449,7 +3512,7 @@
       <c r="C28" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="D28" s="11">
+      <c r="D28" s="13">
         <v>7001</v>
       </c>
     </row>
@@ -3460,21 +3523,21 @@
       <c r="C29" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="D29" s="11">
+      <c r="D29" s="13">
         <v>161</v>
       </c>
     </row>
     <row r="30" s="2" customFormat="1" ht="14.25" spans="4:4">
-      <c r="D30" s="11"/>
+      <c r="D30" s="13"/>
     </row>
     <row r="31" s="2" customFormat="1" ht="14.25" spans="1:5">
-      <c r="A31" s="2" t="s">
+      <c r="A31" s="7" t="s">
         <v>75</v>
       </c>
       <c r="C31" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="D31" s="11" t="s">
+      <c r="D31" s="13" t="s">
         <v>77</v>
       </c>
       <c r="E31" s="2" t="s">
@@ -3482,13 +3545,13 @@
       </c>
     </row>
     <row r="32" s="2" customFormat="1" ht="14.25" spans="1:5">
-      <c r="A32" s="2" t="s">
+      <c r="A32" s="7" t="s">
         <v>79</v>
       </c>
       <c r="C32" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="D32" s="11"/>
+      <c r="D32" s="13"/>
       <c r="E32" s="2" t="s">
         <v>81</v>
       </c>
@@ -3500,7 +3563,7 @@
       <c r="C33" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="D33" s="11"/>
+      <c r="D33" s="13"/>
     </row>
     <row r="34" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A34" s="2" t="s">
@@ -3509,7 +3572,7 @@
       <c r="C34" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="D34" s="11"/>
+      <c r="D34" s="13"/>
       <c r="E34" s="2" t="s">
         <v>86</v>
       </c>
@@ -3521,7 +3584,7 @@
       <c r="C35" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="D35" s="11">
+      <c r="D35" s="13">
         <v>1433</v>
       </c>
     </row>
@@ -3532,7 +3595,7 @@
       <c r="C36" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="D36" s="11">
+      <c r="D36" s="13">
         <v>445</v>
       </c>
       <c r="E36" s="2" t="s">
@@ -3546,13 +3609,13 @@
       <c r="C37" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="D37" s="11"/>
+      <c r="D37" s="13"/>
       <c r="E37" s="2" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="38" s="2" customFormat="1" ht="14.25" spans="4:4">
-      <c r="D38" s="11"/>
+      <c r="D38" s="13"/>
     </row>
     <row r="39" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A39" s="2" t="s">
@@ -3561,7 +3624,7 @@
       <c r="C39" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="D39" s="11">
+      <c r="D39" s="13">
         <v>443</v>
       </c>
       <c r="E39" s="2" t="s">
@@ -3575,7 +3638,7 @@
       <c r="C40" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="D40" s="11">
+      <c r="D40" s="13">
         <v>80</v>
       </c>
       <c r="E40" s="2" t="s">
@@ -3589,7 +3652,7 @@
       <c r="C41" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="D41" s="11" t="s">
+      <c r="D41" s="13" t="s">
         <v>103</v>
       </c>
       <c r="E41" s="2" t="s">
@@ -3603,7 +3666,7 @@
       <c r="C42" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="D42" s="11" t="s">
+      <c r="D42" s="13" t="s">
         <v>103</v>
       </c>
       <c r="E42" s="2" t="s">
@@ -3617,7 +3680,7 @@
       <c r="C43" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="D43" s="11" t="s">
+      <c r="D43" s="13" t="s">
         <v>103</v>
       </c>
       <c r="E43" s="2" t="s">
@@ -3631,7 +3694,7 @@
       <c r="C44" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="D44" s="11" t="s">
+      <c r="D44" s="13" t="s">
         <v>113</v>
       </c>
       <c r="E44" s="2" t="s">
@@ -3645,7 +3708,7 @@
       <c r="C45" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="D45" s="11">
+      <c r="D45" s="13">
         <v>443</v>
       </c>
       <c r="E45" s="2" t="s">
@@ -3659,7 +3722,7 @@
       <c r="C46" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="D46" s="11">
+      <c r="D46" s="13">
         <v>443</v>
       </c>
       <c r="E46" s="2" t="s">
@@ -3673,7 +3736,7 @@
       <c r="C47" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="D47" s="11">
+      <c r="D47" s="13">
         <v>443</v>
       </c>
       <c r="E47" s="2" t="s">
@@ -3687,7 +3750,7 @@
       <c r="C48" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="D48" s="11">
+      <c r="D48" s="13">
         <v>9100</v>
       </c>
       <c r="E48" s="2" t="s">
@@ -3695,7 +3758,7 @@
       </c>
     </row>
     <row r="49" s="2" customFormat="1" ht="14.25" spans="4:4">
-      <c r="D49" s="11"/>
+      <c r="D49" s="13"/>
     </row>
     <row r="50" s="2" customFormat="1" ht="14.25" spans="1:4">
       <c r="A50" s="2" t="s">
@@ -3704,7 +3767,7 @@
       <c r="C50" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="D50" s="11" t="s">
+      <c r="D50" s="13" t="s">
         <v>35</v>
       </c>
     </row>
@@ -3715,7 +3778,7 @@
       <c r="C51" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="D51" s="11" t="s">
+      <c r="D51" s="13" t="s">
         <v>35</v>
       </c>
     </row>
@@ -3726,7 +3789,7 @@
       <c r="C52" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="D52" s="11" t="s">
+      <c r="D52" s="13" t="s">
         <v>35</v>
       </c>
     </row>
@@ -3737,12 +3800,27 @@
       <c r="C53" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="D53" s="11"/>
+      <c r="D53" s="13"/>
     </row>
     <row r="54" s="2" customFormat="1" ht="14.25" spans="4:4">
-      <c r="D54" s="11"/>
+      <c r="D54" s="13"/>
+    </row>
+    <row r="56" s="15" customFormat="1" ht="25.5" spans="1:4">
+      <c r="A56" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="D56" s="3"/>
+    </row>
+    <row r="57" s="15" customFormat="1" ht="25.5" spans="4:4">
+      <c r="D57" s="3"/>
+    </row>
+    <row r="58" s="15" customFormat="1" ht="25.5" spans="4:4">
+      <c r="D58" s="3"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A56:XFD58"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555556" footer="0.511805555555556"/>
   <headerFooter/>
 </worksheet>
@@ -3751,8 +3829,8 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr/>
-  <dimension ref="A1:E21"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="4"/>
+  <dimension ref="A1:XFD27"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="16.5" customWidth="1"/>
     <col min="2" max="2" width="5.625" customWidth="1"/>
@@ -3768,7 +3846,7 @@
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="4" t="s">
         <v>2</v>
       </c>
       <c r="E1" s="1" t="s">
@@ -3777,159 +3855,169 @@
     </row>
     <row r="3" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A3" s="2" t="s">
-        <v>666</v>
+        <v>677</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>667</v>
+        <v>678</v>
       </c>
     </row>
     <row r="4" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A4" s="2" t="s">
-        <v>668</v>
+        <v>679</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>669</v>
+        <v>680</v>
       </c>
     </row>
     <row r="5" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A5" s="2" t="s">
-        <v>670</v>
+        <v>681</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>671</v>
+        <v>682</v>
       </c>
     </row>
     <row r="6" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A6" s="2" t="s">
-        <v>672</v>
+        <v>683</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>673</v>
+        <v>684</v>
       </c>
     </row>
     <row r="7" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A7" s="2" t="s">
-        <v>674</v>
+        <v>685</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>675</v>
+        <v>686</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>676</v>
+        <v>687</v>
       </c>
     </row>
     <row r="8" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A8" s="2" t="s">
-        <v>677</v>
+        <v>688</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>678</v>
+        <v>689</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>679</v>
+        <v>690</v>
       </c>
     </row>
     <row r="9" s="2" customFormat="1" ht="14.25"/>
     <row r="10" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A10" s="2" t="s">
-        <v>531</v>
+        <v>542</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>532</v>
+        <v>543</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>533</v>
+        <v>544</v>
       </c>
     </row>
     <row r="11" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A11" s="2" t="s">
-        <v>534</v>
+        <v>545</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>535</v>
+        <v>546</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>536</v>
+        <v>547</v>
       </c>
     </row>
     <row r="12" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A12" s="2" t="s">
-        <v>537</v>
+        <v>548</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>538</v>
+        <v>549</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>539</v>
+        <v>550</v>
       </c>
     </row>
     <row r="13" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A13" s="2" t="s">
-        <v>540</v>
+        <v>551</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>541</v>
+        <v>552</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>540</v>
+        <v>551</v>
       </c>
     </row>
     <row r="14" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A14" s="2" t="s">
-        <v>542</v>
+        <v>553</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>543</v>
+        <v>554</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>544</v>
+        <v>555</v>
       </c>
     </row>
     <row r="15" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A15" s="2" t="s">
-        <v>545</v>
+        <v>556</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>546</v>
+        <v>557</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>547</v>
+        <v>558</v>
       </c>
     </row>
     <row r="16" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A16" s="2" t="s">
-        <v>548</v>
+        <v>559</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>549</v>
+        <v>560</v>
       </c>
     </row>
     <row r="18" customFormat="1"/>
     <row r="19" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A19" s="2" t="s">
-        <v>589</v>
+        <v>600</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>590</v>
+        <v>601</v>
       </c>
     </row>
     <row r="20" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A20" s="2" t="s">
-        <v>616</v>
+        <v>627</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>617</v>
+        <v>628</v>
       </c>
     </row>
     <row r="21" s="2" customFormat="1" ht="156.75" spans="1:3">
       <c r="A21" s="2" t="s">
-        <v>310</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>311</v>
-      </c>
-    </row>
+        <v>313</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="25" s="3" customFormat="1" ht="25.5" spans="1:1">
+      <c r="A25" s="6" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="26" s="3" customFormat="1" ht="25.5"/>
+    <row r="27" s="3" customFormat="1" ht="25.5"/>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A25:XFD27"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555556" footer="0.511805555555556"/>
   <headerFooter/>
 </worksheet>
@@ -3938,8 +4026,8 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr/>
-  <dimension ref="A1:E26"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="4"/>
+  <dimension ref="A1:XFD32"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
     <col min="2" max="2" width="8.625" customWidth="1"/>
@@ -3955,7 +4043,7 @@
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="4" t="s">
         <v>2</v>
       </c>
       <c r="E1" s="1" t="s">
@@ -3964,53 +4052,53 @@
     </row>
     <row r="3" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A3" s="2" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="4" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A4" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="5" s="2" customFormat="1" ht="14.25" spans="1:5">
-      <c r="A5" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="C5" s="2" t="s">
+    </row>
+    <row r="5" s="2" customFormat="1" ht="14.25" spans="1:3">
+      <c r="A5" s="7" t="s">
         <v>139</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="C5" s="7" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="6" s="2" customFormat="1" ht="14.25" spans="1:3">
+    <row r="6" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A6" s="2" t="s">
         <v>141</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>142</v>
       </c>
+      <c r="E6" s="2" t="s">
+        <v>143</v>
+      </c>
     </row>
     <row r="7" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A7" s="2" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
     </row>
     <row r="8" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A8" s="2" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>145</v>
@@ -4018,103 +4106,100 @@
     </row>
     <row r="9" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A9" s="2" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="10" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A10" s="2" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="11" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A11" s="2" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="12" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A12" s="2" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="13" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A13" s="2" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="14" s="2" customFormat="1" ht="14.25" spans="1:5">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="14" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A14" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>157</v>
-      </c>
-      <c r="E14" s="2" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="15" s="2" customFormat="1" ht="14.25" spans="1:3">
+    <row r="15" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A15" s="2" t="s">
         <v>159</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>160</v>
       </c>
+      <c r="E15" s="2" t="s">
+        <v>161</v>
+      </c>
     </row>
     <row r="16" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A16" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="17" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A17" s="2" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="18" s="2" customFormat="1" ht="144" customHeight="1" spans="1:3">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="18" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A18" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="C18" s="4" t="s">
         <v>166</v>
       </c>
-    </row>
-    <row r="19" s="2" customFormat="1" ht="14.25" spans="1:3">
+      <c r="C18" s="2" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="19" s="2" customFormat="1" ht="144" customHeight="1" spans="1:3">
       <c r="A19" s="2" t="s">
-        <v>167</v>
-      </c>
-      <c r="C19" s="2" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="20" s="2" customFormat="1" ht="14.25" spans="1:5">
+      <c r="C19" s="5" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="20" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A20" s="2" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="E20" s="2" t="s">
         <v>171</v>
       </c>
     </row>
@@ -4129,33 +4214,54 @@
         <v>174</v>
       </c>
     </row>
-    <row r="22" s="2" customFormat="1" ht="70" customHeight="1" spans="1:3">
+    <row r="22" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A22" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="C22" s="4" t="s">
+      <c r="C22" s="2" t="s">
         <v>176</v>
       </c>
-    </row>
-    <row r="23" s="2" customFormat="1" ht="14.25" spans="1:3">
+      <c r="E22" s="2" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="23" s="2" customFormat="1" ht="70" customHeight="1" spans="1:3">
       <c r="A23" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="C23" s="2" t="s">
         <v>178</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>179</v>
       </c>
     </row>
     <row r="24" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A24" s="2" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="25" s="2" customFormat="1" ht="14.25"/>
+        <v>181</v>
+      </c>
+    </row>
+    <row r="25" s="2" customFormat="1" ht="14.25" spans="1:3">
+      <c r="A25" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>183</v>
+      </c>
+    </row>
     <row r="26" s="2" customFormat="1" ht="14.25"/>
+    <row r="27" s="2" customFormat="1" ht="14.25"/>
+    <row r="30" s="3" customFormat="1" ht="25.5" spans="1:1">
+      <c r="A30" s="6" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="31" s="3" customFormat="1" ht="25.5"/>
+    <row r="32" s="3" customFormat="1" ht="25.5"/>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A30:XFD32"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555556" footer="0.511805555555556"/>
   <headerFooter/>
 </worksheet>
@@ -4164,12 +4270,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr/>
-  <dimension ref="A1:E41"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="4"/>
+  <dimension ref="A1:XFD46"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="21.5" customWidth="1"/>
     <col min="3" max="3" width="47.375" customWidth="1"/>
-    <col min="4" max="4" width="12.875" style="10" customWidth="1"/>
+    <col min="4" max="4" width="12.875" style="12" customWidth="1"/>
     <col min="5" max="5" width="52.625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -4180,7 +4286,7 @@
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="4" t="s">
         <v>2</v>
       </c>
       <c r="E1" s="1" t="s">
@@ -4189,377 +4295,387 @@
     </row>
     <row r="3" s="2" customFormat="1" ht="14.25" spans="1:4">
       <c r="A3" s="2" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>182</v>
-      </c>
-      <c r="D3" s="11"/>
+        <v>185</v>
+      </c>
+      <c r="D3" s="13"/>
     </row>
     <row r="4" s="2" customFormat="1" ht="14.25" spans="1:4">
       <c r="A4" s="2" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>182</v>
-      </c>
-      <c r="D4" s="11"/>
+        <v>185</v>
+      </c>
+      <c r="D4" s="13"/>
     </row>
     <row r="5" s="2" customFormat="1" ht="85" customHeight="1" spans="1:4">
       <c r="A5" s="2" t="s">
-        <v>184</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>185</v>
-      </c>
-      <c r="D5" s="11"/>
+        <v>187</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="D5" s="13"/>
     </row>
     <row r="6" s="2" customFormat="1" ht="14.25" spans="4:4">
-      <c r="D6" s="11"/>
+      <c r="D6" s="13"/>
     </row>
     <row r="7" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A7" s="2" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>187</v>
-      </c>
-      <c r="D7" s="11"/>
+        <v>190</v>
+      </c>
+      <c r="D7" s="13"/>
       <c r="E7" s="2" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
     </row>
     <row r="8" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A8" s="2" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>190</v>
-      </c>
-      <c r="D8" s="11"/>
+        <v>193</v>
+      </c>
+      <c r="D8" s="13"/>
       <c r="E8" s="2" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
     </row>
     <row r="9" s="2" customFormat="1" ht="14.25" spans="1:4">
       <c r="A9" s="2" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>193</v>
-      </c>
-      <c r="D9" s="11"/>
+        <v>196</v>
+      </c>
+      <c r="D9" s="13"/>
     </row>
     <row r="10" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A10" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="D10" s="11"/>
+        <v>198</v>
+      </c>
+      <c r="D10" s="13"/>
       <c r="E10" s="2" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
     </row>
     <row r="11" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A11" s="2" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="D11" s="11"/>
+        <v>198</v>
+      </c>
+      <c r="D11" s="13"/>
       <c r="E11" s="2" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
     </row>
     <row r="12" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A12" s="2" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>200</v>
-      </c>
-      <c r="D12" s="11"/>
+        <v>203</v>
+      </c>
+      <c r="D12" s="13"/>
       <c r="E12" s="2" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
     </row>
     <row r="13" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A13" s="2" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="D13" s="11"/>
+        <v>206</v>
+      </c>
+      <c r="D13" s="13"/>
       <c r="E13" s="2" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
     </row>
     <row r="14" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A14" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>206</v>
-      </c>
-      <c r="D14" s="11"/>
+        <v>209</v>
+      </c>
+      <c r="D14" s="13"/>
       <c r="E14" s="2" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
     </row>
     <row r="15" s="2" customFormat="1" ht="14.25" spans="1:4">
       <c r="A15" s="2" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>209</v>
-      </c>
-      <c r="D15" s="11"/>
+        <v>212</v>
+      </c>
+      <c r="D15" s="13"/>
     </row>
     <row r="16" s="2" customFormat="1" ht="14.25" spans="4:4">
-      <c r="D16" s="11"/>
+      <c r="D16" s="13"/>
     </row>
     <row r="17" s="2" customFormat="1" ht="14.25" spans="1:4">
       <c r="A17" s="2" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>211</v>
-      </c>
-      <c r="D17" s="11"/>
+        <v>214</v>
+      </c>
+      <c r="D17" s="13"/>
     </row>
     <row r="18" s="2" customFormat="1" ht="14.25" spans="1:4">
       <c r="A18" s="2" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>213</v>
-      </c>
-      <c r="D18" s="11"/>
+        <v>216</v>
+      </c>
+      <c r="D18" s="13"/>
     </row>
     <row r="19" s="2" customFormat="1" ht="14.25" spans="1:4">
       <c r="A19" s="2" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>215</v>
-      </c>
-      <c r="D19" s="11"/>
+        <v>218</v>
+      </c>
+      <c r="D19" s="13"/>
     </row>
     <row r="20" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A20" s="2" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="D20" s="11"/>
+        <v>220</v>
+      </c>
+      <c r="D20" s="13"/>
       <c r="E20" s="2" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
     </row>
     <row r="21" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A21" s="2" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>220</v>
-      </c>
-      <c r="D21" s="11"/>
+        <v>223</v>
+      </c>
+      <c r="D21" s="13"/>
       <c r="E21" s="2" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
     </row>
     <row r="22" s="2" customFormat="1" ht="14.25" spans="1:4">
       <c r="A22" s="2" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>223</v>
-      </c>
-      <c r="D22" s="11"/>
+        <v>226</v>
+      </c>
+      <c r="D22" s="13"/>
     </row>
     <row r="23" s="2" customFormat="1" ht="14.25" spans="1:4">
       <c r="A23" s="2" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>225</v>
-      </c>
-      <c r="D23" s="11"/>
+        <v>228</v>
+      </c>
+      <c r="D23" s="13"/>
     </row>
     <row r="24" s="2" customFormat="1" ht="14.25" spans="1:4">
       <c r="A24" s="2" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>227</v>
-      </c>
-      <c r="D24" s="11"/>
+        <v>230</v>
+      </c>
+      <c r="D24" s="13"/>
     </row>
     <row r="25" s="2" customFormat="1" ht="14.25" spans="1:4">
       <c r="A25" s="2" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>229</v>
-      </c>
-      <c r="D25" s="11"/>
+        <v>232</v>
+      </c>
+      <c r="D25" s="13"/>
     </row>
     <row r="26" s="2" customFormat="1" ht="14.25" spans="4:4">
-      <c r="D26" s="11"/>
+      <c r="D26" s="13"/>
     </row>
     <row r="27" s="2" customFormat="1" ht="213.75" spans="1:4">
       <c r="A27" s="2" t="s">
-        <v>230</v>
-      </c>
-      <c r="C27" s="4" t="s">
-        <v>231</v>
-      </c>
-      <c r="D27" s="11"/>
+        <v>233</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>234</v>
+      </c>
+      <c r="D27" s="13"/>
     </row>
     <row r="28" s="2" customFormat="1" ht="14.25" spans="1:4">
       <c r="A28" s="2" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>233</v>
-      </c>
-      <c r="D28" s="11"/>
+        <v>236</v>
+      </c>
+      <c r="D28" s="13"/>
     </row>
     <row r="29" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A29" s="2" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>235</v>
-      </c>
-      <c r="D29" s="11"/>
+        <v>238</v>
+      </c>
+      <c r="D29" s="13"/>
       <c r="E29" s="2" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
     </row>
     <row r="30" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A30" s="2" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="D30" s="11"/>
+        <v>241</v>
+      </c>
+      <c r="D30" s="13"/>
       <c r="E30" s="2" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
     </row>
     <row r="31" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A31" s="2" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>241</v>
-      </c>
-      <c r="D31" s="11"/>
+        <v>244</v>
+      </c>
+      <c r="D31" s="13"/>
       <c r="E31" s="2" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
     </row>
     <row r="32" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A32" s="2" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>244</v>
-      </c>
-      <c r="D32" s="11"/>
+        <v>247</v>
+      </c>
+      <c r="D32" s="13"/>
       <c r="E32" s="2" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="33" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A33" s="2" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>247</v>
-      </c>
-      <c r="D33" s="11"/>
+        <v>250</v>
+      </c>
+      <c r="D33" s="13"/>
       <c r="E33" s="2" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
     </row>
     <row r="34" s="2" customFormat="1" ht="14.25" spans="1:4">
       <c r="A34" s="2" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>250</v>
-      </c>
-      <c r="D34" s="11"/>
+        <v>253</v>
+      </c>
+      <c r="D34" s="13"/>
     </row>
     <row r="35" s="2" customFormat="1" ht="14.25" spans="1:4">
       <c r="A35" s="2" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>252</v>
-      </c>
-      <c r="D35" s="11"/>
+        <v>255</v>
+      </c>
+      <c r="D35" s="13"/>
     </row>
     <row r="36" s="2" customFormat="1" ht="57" spans="1:4">
       <c r="A36" s="2" t="s">
-        <v>253</v>
-      </c>
-      <c r="C36" s="4" t="s">
-        <v>254</v>
-      </c>
-      <c r="D36" s="11"/>
+        <v>256</v>
+      </c>
+      <c r="C36" s="5" t="s">
+        <v>257</v>
+      </c>
+      <c r="D36" s="13"/>
     </row>
     <row r="37" s="2" customFormat="1" ht="14.25" spans="1:4">
       <c r="A37" s="2" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>256</v>
-      </c>
-      <c r="D37" s="11"/>
+        <v>259</v>
+      </c>
+      <c r="D37" s="13"/>
     </row>
     <row r="38" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A38" s="2" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>258</v>
-      </c>
-      <c r="D38" s="11"/>
+        <v>261</v>
+      </c>
+      <c r="D38" s="13"/>
       <c r="E38" s="2" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
     </row>
     <row r="39" s="2" customFormat="1" ht="14.25" spans="4:4">
-      <c r="D39" s="11"/>
+      <c r="D39" s="13"/>
     </row>
     <row r="40" s="2" customFormat="1" ht="14.25" spans="1:4">
       <c r="A40" s="2" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>261</v>
-      </c>
-      <c r="D40" s="11"/>
+        <v>264</v>
+      </c>
+      <c r="D40" s="13"/>
     </row>
     <row r="41" s="2" customFormat="1" ht="14.25" spans="1:4">
       <c r="A41" s="2" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>263</v>
-      </c>
-      <c r="D41" s="11"/>
-    </row>
+        <v>266</v>
+      </c>
+      <c r="D41" s="13"/>
+    </row>
+    <row r="44" s="3" customFormat="1" ht="25.5" spans="1:1">
+      <c r="A44" s="6" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="45" s="3" customFormat="1" ht="25.5"/>
+    <row r="46" s="3" customFormat="1" ht="25.5"/>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A44:XFD46"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555556" footer="0.511805555555556"/>
   <headerFooter/>
 </worksheet>
@@ -4568,8 +4684,8 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr/>
-  <dimension ref="A1:E31"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="4"/>
+  <dimension ref="A1:XFD32"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="18.25" customWidth="1"/>
     <col min="2" max="2" width="5.75" customWidth="1"/>
@@ -4585,7 +4701,7 @@
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="4" t="s">
         <v>2</v>
       </c>
       <c r="E1" s="1" t="s">
@@ -4594,241 +4710,249 @@
     </row>
     <row r="3" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A3" s="2" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
     </row>
     <row r="4" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A4" s="2" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
     </row>
     <row r="5" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A5" s="2" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
     </row>
     <row r="6" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A6" s="2" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
     </row>
     <row r="7" s="2" customFormat="1" ht="15" customHeight="1" spans="1:5">
       <c r="A7" s="2" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>276</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>277</v>
+        <v>279</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>280</v>
       </c>
     </row>
     <row r="8" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A8" s="2" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
     </row>
     <row r="9" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A9" s="2" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
     </row>
     <row r="10" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A10" s="2" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
     </row>
     <row r="11" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A11" s="2" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
     </row>
     <row r="12" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A12" s="2" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
     </row>
     <row r="13" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A13" s="2" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
     </row>
     <row r="14" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A14" s="2" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
     </row>
     <row r="15" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A15" s="2" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
     </row>
     <row r="16" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A16" s="2" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
     </row>
     <row r="17" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A17" s="2" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
     </row>
     <row r="18" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A18" s="2" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
     </row>
     <row r="19" s="2" customFormat="1" ht="48" customHeight="1" spans="1:3">
       <c r="A19" s="2" t="s">
-        <v>306</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>307</v>
+        <v>309</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>310</v>
       </c>
     </row>
     <row r="20" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A20" s="2" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
     </row>
     <row r="21" s="2" customFormat="1" ht="148" customHeight="1" spans="1:3">
       <c r="A21" s="2" t="s">
-        <v>310</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>311</v>
+        <v>313</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>314</v>
       </c>
     </row>
     <row r="22" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A22" s="2" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
     </row>
     <row r="23" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A23" s="2" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
     </row>
     <row r="24" s="2" customFormat="1" ht="14.25"/>
     <row r="25" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A25" s="2" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
     </row>
     <row r="26" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A26" s="2" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
     </row>
     <row r="27" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A27" s="2" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
     </row>
     <row r="28" s="2" customFormat="1" ht="14.25"/>
     <row r="29" s="2" customFormat="1" ht="14.25"/>
-    <row r="30" s="2" customFormat="1" ht="14.25"/>
-    <row r="31" s="2" customFormat="1" ht="14.25"/>
+    <row r="30" s="3" customFormat="1" ht="25.5" spans="1:1">
+      <c r="A30" s="6" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="31" s="3" customFormat="1" ht="25.5"/>
+    <row r="32" s="3" customFormat="1" ht="25.5"/>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A30:XFD32"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555556" footer="0.511805555555556"/>
   <headerFooter/>
 </worksheet>
@@ -4837,10 +4961,10 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr/>
-  <dimension ref="A1:E29"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="4"/>
+  <dimension ref="A1:XFD37"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
-    <col min="1" max="1" width="19.375" customWidth="1"/>
+    <col min="1" max="1" width="21.5" customWidth="1"/>
     <col min="3" max="3" width="73.75" customWidth="1"/>
     <col min="4" max="4" width="14" customWidth="1"/>
     <col min="5" max="5" width="37.75" customWidth="1"/>
@@ -4853,7 +4977,7 @@
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="4" t="s">
         <v>2</v>
       </c>
       <c r="E1" s="1" t="s">
@@ -4862,199 +4986,220 @@
     </row>
     <row r="3" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A3" s="2" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
     </row>
     <row r="4" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A4" s="2" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
     </row>
     <row r="5" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A5" s="2" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>331</v>
-      </c>
-    </row>
-    <row r="6" s="9" customFormat="1" ht="14.25" spans="1:3">
-      <c r="A6" s="9" t="s">
-        <v>332</v>
-      </c>
-      <c r="C6" s="9" t="s">
-        <v>333</v>
+        <v>334</v>
+      </c>
+    </row>
+    <row r="6" s="11" customFormat="1" ht="14.25" spans="1:3">
+      <c r="A6" s="11" t="s">
+        <v>335</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>336</v>
       </c>
     </row>
     <row r="7" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A7" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>334</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>331</v>
       </c>
     </row>
     <row r="8" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A8" s="2" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
     </row>
     <row r="9" s="2" customFormat="1" ht="14.25"/>
     <row r="10" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A10" s="2" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
     </row>
     <row r="11" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A11" s="2" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
     </row>
     <row r="12" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A12" s="2" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
     </row>
     <row r="13" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A13" s="2" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
     </row>
     <row r="14" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A14" s="2" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
     </row>
     <row r="15" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A15" s="2" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
     </row>
     <row r="16" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A16" s="2" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
     </row>
     <row r="17" s="2" customFormat="1" ht="14.25"/>
     <row r="18" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A18" s="2" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
     </row>
     <row r="19" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A19" s="2" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
     </row>
     <row r="20" s="2" customFormat="1" ht="90" customHeight="1" spans="1:3">
       <c r="A20" s="2" t="s">
-        <v>356</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>357</v>
+        <v>359</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>360</v>
       </c>
     </row>
     <row r="21" s="2" customFormat="1" ht="14.25"/>
-    <row r="22" s="2" customFormat="1" ht="14.25" spans="1:3">
-      <c r="A22" s="2" t="s">
-        <v>358</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>359</v>
+    <row r="22" s="2" customFormat="1" ht="14.25" spans="1:5">
+      <c r="A22" s="7" t="s">
+        <v>361</v>
+      </c>
+      <c r="C22" s="7" t="s">
+        <v>362</v>
+      </c>
+      <c r="E22" s="7" t="s">
+        <v>363</v>
       </c>
     </row>
     <row r="23" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A23" s="2" t="s">
-        <v>360</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>361</v>
+        <v>364</v>
+      </c>
+      <c r="C23" s="7" t="s">
+        <v>365</v>
       </c>
     </row>
     <row r="24" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A24" s="2" t="s">
-        <v>362</v>
+        <v>366</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
     </row>
     <row r="25" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A25" s="2" t="s">
-        <v>364</v>
+        <v>368</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>365</v>
+        <v>369</v>
       </c>
     </row>
     <row r="26" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A26" s="2" t="s">
-        <v>366</v>
+        <v>370</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>367</v>
+        <v>371</v>
       </c>
     </row>
     <row r="27" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A27" s="2" t="s">
-        <v>368</v>
-      </c>
-      <c r="C27" s="8" t="s">
-        <v>369</v>
-      </c>
-    </row>
-    <row r="28" s="2" customFormat="1" ht="14.25"/>
-    <row r="29" s="2" customFormat="1" ht="85" customHeight="1" spans="1:3">
-      <c r="A29" s="2" t="s">
-        <v>184</v>
-      </c>
-      <c r="C29" s="4" t="s">
-        <v>185</v>
-      </c>
-    </row>
+        <v>372</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="28" s="2" customFormat="1" ht="14.25" spans="1:3">
+      <c r="A28" s="2" t="s">
+        <v>374</v>
+      </c>
+      <c r="C28" s="7" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="29" s="2" customFormat="1" ht="14.25"/>
+    <row r="30" s="2" customFormat="1" ht="85" customHeight="1" spans="1:3">
+      <c r="A30" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="35" s="3" customFormat="1" ht="25.5" spans="1:1">
+      <c r="A35" s="6" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="36" s="3" customFormat="1" ht="25.5"/>
+    <row r="37" s="3" customFormat="1" ht="25.5"/>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A35:XFD37"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555556" footer="0.511805555555556"/>
   <headerFooter/>
 </worksheet>
@@ -5063,8 +5208,8 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr/>
-  <dimension ref="A1:E49"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="4"/>
+  <dimension ref="A1:XFD49"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="18.25" customWidth="1"/>
     <col min="3" max="3" width="50.25" customWidth="1"/>
@@ -5079,7 +5224,7 @@
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="4" t="s">
         <v>2</v>
       </c>
       <c r="E1" s="1" t="s">
@@ -5088,277 +5233,281 @@
     </row>
     <row r="3" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A3" s="2" t="s">
-        <v>370</v>
+        <v>376</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>371</v>
+        <v>377</v>
       </c>
     </row>
     <row r="4" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A4" s="2" t="s">
-        <v>372</v>
+        <v>378</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>373</v>
+        <v>379</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>374</v>
+        <v>380</v>
       </c>
     </row>
     <row r="5" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A5" s="2" t="s">
-        <v>375</v>
+        <v>381</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>376</v>
+        <v>382</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>377</v>
+        <v>383</v>
       </c>
     </row>
     <row r="6" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A6" s="2" t="s">
-        <v>378</v>
+        <v>384</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>379</v>
+        <v>385</v>
       </c>
     </row>
     <row r="7" s="2" customFormat="1" ht="14.25"/>
     <row r="8" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A8" s="2" t="s">
-        <v>380</v>
+        <v>386</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>381</v>
+        <v>387</v>
       </c>
     </row>
     <row r="9" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A9" s="2" t="s">
-        <v>382</v>
+        <v>388</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>383</v>
+        <v>389</v>
       </c>
     </row>
     <row r="10" s="2" customFormat="1" ht="14.25"/>
     <row r="11" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A11" s="2" t="s">
-        <v>384</v>
+        <v>390</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>385</v>
+        <v>391</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>386</v>
+        <v>392</v>
       </c>
     </row>
     <row r="12" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A12" s="2" t="s">
-        <v>387</v>
+        <v>393</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>388</v>
+        <v>394</v>
       </c>
     </row>
     <row r="13" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A13" s="2" t="s">
-        <v>389</v>
+        <v>395</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>390</v>
+        <v>396</v>
       </c>
     </row>
     <row r="14" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A14" s="2" t="s">
-        <v>391</v>
+        <v>397</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>392</v>
+        <v>398</v>
       </c>
     </row>
     <row r="15" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A15" s="2" t="s">
-        <v>393</v>
+        <v>399</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>394</v>
+        <v>400</v>
       </c>
     </row>
     <row r="16" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A16" s="2" t="s">
-        <v>395</v>
+        <v>401</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>396</v>
+        <v>402</v>
       </c>
     </row>
     <row r="17" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A17" s="2" t="s">
-        <v>397</v>
+        <v>403</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>398</v>
+        <v>404</v>
       </c>
     </row>
     <row r="18" s="2" customFormat="1" ht="14.25"/>
     <row r="19" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A19" s="2" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
     </row>
     <row r="20" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A20" s="2" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
     </row>
     <row r="21" s="2" customFormat="1" ht="85" customHeight="1" spans="1:3">
       <c r="A21" s="2" t="s">
-        <v>184</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>185</v>
+        <v>187</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>188</v>
       </c>
     </row>
     <row r="22" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A22" s="2" t="s">
-        <v>399</v>
+        <v>405</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>400</v>
+        <v>406</v>
       </c>
     </row>
     <row r="23" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A23" s="2" t="s">
-        <v>401</v>
+        <v>407</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>402</v>
+        <v>408</v>
       </c>
     </row>
     <row r="24" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A24" s="2" t="s">
-        <v>403</v>
+        <v>409</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>404</v>
+        <v>410</v>
       </c>
     </row>
     <row r="25" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A25" s="2" t="s">
-        <v>405</v>
+        <v>411</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>406</v>
+        <v>412</v>
       </c>
     </row>
     <row r="26" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A26" s="2" t="s">
-        <v>407</v>
+        <v>413</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>406</v>
+        <v>412</v>
       </c>
     </row>
     <row r="27" s="2" customFormat="1" ht="66" customHeight="1" spans="1:3">
       <c r="A27" s="2" t="s">
-        <v>408</v>
-      </c>
-      <c r="C27" s="4" t="s">
-        <v>409</v>
+        <v>414</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>415</v>
       </c>
     </row>
     <row r="28" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A28" s="2" t="s">
-        <v>410</v>
+        <v>416</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>411</v>
+        <v>417</v>
       </c>
     </row>
     <row r="29" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A29" s="2" t="s">
-        <v>412</v>
+        <v>418</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>413</v>
+        <v>419</v>
       </c>
     </row>
     <row r="30" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A30" s="2" t="s">
-        <v>414</v>
+        <v>420</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>415</v>
+        <v>421</v>
       </c>
     </row>
     <row r="31" s="2" customFormat="1" ht="14.25"/>
     <row r="32" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A32" s="2" t="s">
-        <v>416</v>
-      </c>
-      <c r="C32" s="8" t="s">
-        <v>417</v>
+        <v>422</v>
+      </c>
+      <c r="C32" s="7" t="s">
+        <v>423</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>418</v>
+        <v>424</v>
       </c>
     </row>
     <row r="33" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A33" s="2" t="s">
-        <v>419</v>
+        <v>425</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>420</v>
+        <v>426</v>
       </c>
     </row>
     <row r="34" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A34" s="2" t="s">
-        <v>421</v>
-      </c>
-      <c r="C34" s="8" t="s">
-        <v>422</v>
+        <v>427</v>
+      </c>
+      <c r="C34" s="7" t="s">
+        <v>428</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>423</v>
+        <v>429</v>
       </c>
     </row>
     <row r="35" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A35" s="2" t="s">
-        <v>424</v>
+        <v>430</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>425</v>
+        <v>431</v>
       </c>
     </row>
     <row r="36" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A36" s="2" t="s">
-        <v>426</v>
+        <v>432</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>427</v>
+        <v>433</v>
       </c>
     </row>
     <row r="37" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A37" s="2" t="s">
-        <v>428</v>
+        <v>434</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>429</v>
+        <v>435</v>
       </c>
     </row>
     <row r="38" s="2" customFormat="1" ht="14.25"/>
     <row r="39" s="2" customFormat="1" ht="14.25"/>
     <row r="40" s="2" customFormat="1" ht="14.25"/>
-    <row r="41" s="2" customFormat="1" ht="14.25"/>
-    <row r="42" s="2" customFormat="1" ht="14.25"/>
-    <row r="43" s="2" customFormat="1" ht="14.25"/>
+    <row r="41" s="3" customFormat="1" ht="25.5" spans="1:1">
+      <c r="A41" s="6" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="42" s="3" customFormat="1" ht="25.5"/>
+    <row r="43" s="3" customFormat="1" ht="25.5"/>
     <row r="44" s="2" customFormat="1" ht="14.25"/>
     <row r="45" s="2" customFormat="1" ht="14.25"/>
     <row r="46" s="2" customFormat="1" ht="14.25"/>
@@ -5366,6 +5515,9 @@
     <row r="48" s="2" customFormat="1" ht="14.25"/>
     <row r="49" s="2" customFormat="1" ht="14.25"/>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A41:XFD43"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555556" footer="0.511805555555556"/>
   <headerFooter/>
 </worksheet>
@@ -5374,12 +5526,12 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr/>
-  <dimension ref="A1:E29"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="4"/>
+  <dimension ref="A1:XFD37"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="15.625" customWidth="1"/>
     <col min="3" max="3" width="39.375" customWidth="1"/>
-    <col min="4" max="4" width="19.375" style="5" customWidth="1"/>
+    <col min="4" max="4" width="19.375" style="8" customWidth="1"/>
     <col min="5" max="5" width="34.875" customWidth="1"/>
   </cols>
   <sheetData>
@@ -5390,7 +5542,7 @@
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="9" t="s">
         <v>2</v>
       </c>
       <c r="E1" s="1" t="s">
@@ -5399,314 +5551,349 @@
     </row>
     <row r="3" s="2" customFormat="1" ht="14.25" spans="1:4">
       <c r="A3" s="2" t="s">
-        <v>430</v>
+        <v>436</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>431</v>
-      </c>
-      <c r="D3" s="7">
+        <v>437</v>
+      </c>
+      <c r="D3" s="10">
         <v>443</v>
       </c>
     </row>
-    <row r="4" s="2" customFormat="1" ht="14.25" spans="1:4">
-      <c r="A4" s="2" t="s">
-        <v>432</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>433</v>
-      </c>
-      <c r="D4" s="7">
+    <row r="4" s="2" customFormat="1" ht="14.25" spans="1:5">
+      <c r="A4" s="7" t="s">
+        <v>438</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>439</v>
+      </c>
+      <c r="D4" s="10">
         <v>443</v>
       </c>
+      <c r="E4" s="7" t="s">
+        <v>440</v>
+      </c>
     </row>
     <row r="5" s="2" customFormat="1" ht="14.25" spans="1:4">
-      <c r="A5" s="2" t="s">
-        <v>434</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>435</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>436</v>
+      <c r="A5" s="7" t="s">
+        <v>441</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>442</v>
+      </c>
+      <c r="D5" s="10">
+        <v>10443</v>
       </c>
     </row>
     <row r="6" s="2" customFormat="1" ht="14.25" spans="1:4">
       <c r="A6" s="2" t="s">
-        <v>437</v>
+        <v>443</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>438</v>
-      </c>
-      <c r="D6" s="7">
-        <v>135</v>
+        <v>444</v>
+      </c>
+      <c r="D6" s="10">
+        <v>443</v>
       </c>
     </row>
     <row r="7" s="2" customFormat="1" ht="14.25" spans="1:4">
       <c r="A7" s="2" t="s">
-        <v>439</v>
+        <v>445</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>440</v>
-      </c>
-      <c r="D7" s="7">
-        <v>5985</v>
+        <v>446</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>447</v>
       </c>
     </row>
     <row r="8" s="2" customFormat="1" ht="14.25" spans="1:4">
       <c r="A8" s="2" t="s">
-        <v>441</v>
+        <v>448</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>442</v>
-      </c>
-      <c r="D8" s="7">
-        <v>139</v>
+        <v>449</v>
+      </c>
+      <c r="D8" s="10">
+        <v>135</v>
       </c>
     </row>
     <row r="9" s="2" customFormat="1" ht="14.25" spans="1:4">
       <c r="A9" s="2" t="s">
-        <v>443</v>
+        <v>450</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>444</v>
-      </c>
-      <c r="D9" s="7">
+        <v>451</v>
+      </c>
+      <c r="D9" s="10">
+        <v>5985</v>
+      </c>
+    </row>
+    <row r="10" s="2" customFormat="1" ht="14.25" spans="1:4">
+      <c r="A10" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>453</v>
+      </c>
+      <c r="D10" s="10">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="11" s="2" customFormat="1" ht="14.25" spans="1:4">
+      <c r="A11" s="2" t="s">
+        <v>454</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>455</v>
+      </c>
+      <c r="D11" s="10">
         <v>445</v>
       </c>
     </row>
-    <row r="10" s="2" customFormat="1" ht="14.25" spans="1:5">
-      <c r="A10" s="2" t="s">
+    <row r="12" s="2" customFormat="1" ht="14.25" spans="1:5">
+      <c r="A12" s="2" t="s">
+        <v>456</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>457</v>
+      </c>
+      <c r="D12" s="10">
         <v>445</v>
       </c>
-      <c r="C10" s="2" t="s">
-        <v>446</v>
-      </c>
-      <c r="D10" s="7">
-        <v>445</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>447</v>
-      </c>
-    </row>
-    <row r="11" s="2" customFormat="1" ht="14.25" spans="1:5">
-      <c r="A11" s="2" t="s">
-        <v>448</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>449</v>
-      </c>
-      <c r="D11" s="7">
+      <c r="E12" s="2" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="13" s="2" customFormat="1" ht="14.25" spans="1:5">
+      <c r="A13" s="2" t="s">
+        <v>459</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>460</v>
+      </c>
+      <c r="D13" s="10">
         <v>135</v>
       </c>
-      <c r="E11" s="2" t="s">
-        <v>450</v>
-      </c>
-    </row>
-    <row r="12" s="2" customFormat="1" ht="14.25" spans="1:4">
-      <c r="A12" s="2" t="s">
-        <v>451</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>452</v>
-      </c>
-      <c r="D12" s="7">
-        <v>5900</v>
-      </c>
-    </row>
-    <row r="13" s="2" customFormat="1" ht="14.25" spans="1:4">
-      <c r="A13" s="2" t="s">
-        <v>453</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>454</v>
-      </c>
-      <c r="D13" s="7">
-        <v>3306</v>
+      <c r="E13" s="2" t="s">
+        <v>461</v>
       </c>
     </row>
     <row r="14" s="2" customFormat="1" ht="14.25" spans="1:4">
       <c r="A14" s="2" t="s">
-        <v>455</v>
+        <v>462</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>456</v>
-      </c>
-      <c r="D14" s="7">
-        <v>1433</v>
+        <v>463</v>
+      </c>
+      <c r="D14" s="10">
+        <v>5900</v>
       </c>
     </row>
     <row r="15" s="2" customFormat="1" ht="14.25" spans="1:4">
       <c r="A15" s="2" t="s">
-        <v>457</v>
+        <v>464</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>458</v>
-      </c>
-      <c r="D15" s="7">
-        <v>1521</v>
+        <v>465</v>
+      </c>
+      <c r="D15" s="10">
+        <v>3306</v>
       </c>
     </row>
     <row r="16" s="2" customFormat="1" ht="14.25" spans="1:4">
       <c r="A16" s="2" t="s">
-        <v>459</v>
+        <v>466</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>460</v>
-      </c>
-      <c r="D16" s="7">
-        <v>22</v>
+        <v>467</v>
+      </c>
+      <c r="D16" s="10">
+        <v>1433</v>
       </c>
     </row>
     <row r="17" s="2" customFormat="1" ht="14.25" spans="1:4">
       <c r="A17" s="2" t="s">
-        <v>461</v>
+        <v>468</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>462</v>
-      </c>
-      <c r="D17" s="7" t="s">
-        <v>463</v>
-      </c>
-    </row>
-    <row r="18" s="2" customFormat="1" ht="14.25" spans="1:5">
+        <v>469</v>
+      </c>
+      <c r="D17" s="10">
+        <v>1521</v>
+      </c>
+    </row>
+    <row r="18" s="2" customFormat="1" ht="14.25" spans="1:4">
       <c r="A18" s="2" t="s">
-        <v>464</v>
+        <v>470</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>465</v>
-      </c>
-      <c r="D18" s="7" t="s">
-        <v>463</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>466</v>
-      </c>
-    </row>
-    <row r="19" s="2" customFormat="1" ht="14.25" spans="1:5">
+        <v>471</v>
+      </c>
+      <c r="D18" s="10">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="19" s="2" customFormat="1" ht="14.25" spans="1:4">
       <c r="A19" s="2" t="s">
-        <v>467</v>
+        <v>472</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>468</v>
-      </c>
-      <c r="D19" s="7" t="s">
-        <v>463</v>
-      </c>
-      <c r="E19" s="2" t="s">
-        <v>469</v>
-      </c>
-    </row>
-    <row r="20" s="2" customFormat="1" ht="14.25" spans="1:4">
+        <v>473</v>
+      </c>
+      <c r="D19" s="10" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="20" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A20" s="2" t="s">
-        <v>470</v>
+        <v>475</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>471</v>
-      </c>
-      <c r="D20" s="7" t="s">
-        <v>463</v>
-      </c>
-    </row>
-    <row r="21" s="2" customFormat="1" ht="14.25" spans="1:4">
+        <v>476</v>
+      </c>
+      <c r="D20" s="10" t="s">
+        <v>474</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="21" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A21" s="2" t="s">
-        <v>472</v>
+        <v>478</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>473</v>
-      </c>
-      <c r="D21" s="7">
-        <v>23</v>
+        <v>479</v>
+      </c>
+      <c r="D21" s="10" t="s">
+        <v>474</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>480</v>
       </c>
     </row>
     <row r="22" s="2" customFormat="1" ht="14.25" spans="1:4">
       <c r="A22" s="2" t="s">
+        <v>481</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>482</v>
+      </c>
+      <c r="D22" s="10" t="s">
         <v>474</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>475</v>
-      </c>
-      <c r="D22" s="7" t="s">
-        <v>463</v>
       </c>
     </row>
     <row r="23" s="2" customFormat="1" ht="14.25" spans="1:4">
       <c r="A23" s="2" t="s">
-        <v>476</v>
+        <v>483</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>477</v>
-      </c>
-      <c r="D23" s="7" t="s">
-        <v>463</v>
+        <v>484</v>
+      </c>
+      <c r="D23" s="10">
+        <v>23</v>
       </c>
     </row>
     <row r="24" s="2" customFormat="1" ht="14.25" spans="1:4">
       <c r="A24" s="2" t="s">
-        <v>478</v>
+        <v>485</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>479</v>
-      </c>
-      <c r="D24" s="7" t="s">
-        <v>463</v>
+        <v>486</v>
+      </c>
+      <c r="D24" s="10" t="s">
+        <v>474</v>
       </c>
     </row>
     <row r="25" s="2" customFormat="1" ht="14.25" spans="1:4">
       <c r="A25" s="2" t="s">
-        <v>480</v>
+        <v>487</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>481</v>
-      </c>
-      <c r="D25" s="7" t="s">
-        <v>482</v>
+        <v>488</v>
+      </c>
+      <c r="D25" s="10" t="s">
+        <v>474</v>
       </c>
     </row>
     <row r="26" s="2" customFormat="1" ht="14.25" spans="1:4">
       <c r="A26" s="2" t="s">
-        <v>483</v>
+        <v>489</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>484</v>
-      </c>
-      <c r="D26" s="7" t="s">
-        <v>463</v>
+        <v>490</v>
+      </c>
+      <c r="D26" s="10" t="s">
+        <v>474</v>
       </c>
     </row>
     <row r="27" s="2" customFormat="1" ht="14.25" spans="1:4">
       <c r="A27" s="2" t="s">
-        <v>485</v>
+        <v>491</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>486</v>
-      </c>
-      <c r="D27" s="7" t="s">
-        <v>463</v>
+        <v>492</v>
+      </c>
+      <c r="D27" s="10" t="s">
+        <v>493</v>
       </c>
     </row>
     <row r="28" s="2" customFormat="1" ht="14.25" spans="1:4">
       <c r="A28" s="2" t="s">
-        <v>487</v>
+        <v>494</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>488</v>
-      </c>
-      <c r="D28" s="7" t="s">
-        <v>463</v>
+        <v>495</v>
+      </c>
+      <c r="D28" s="10" t="s">
+        <v>474</v>
       </c>
     </row>
     <row r="29" s="2" customFormat="1" ht="14.25" spans="1:4">
       <c r="A29" s="2" t="s">
-        <v>489</v>
+        <v>496</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>490</v>
-      </c>
-      <c r="D29" s="7">
+        <v>497</v>
+      </c>
+      <c r="D29" s="10" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="30" s="2" customFormat="1" ht="14.25" spans="1:4">
+      <c r="A30" s="2" t="s">
+        <v>498</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>499</v>
+      </c>
+      <c r="D30" s="10" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="31" s="2" customFormat="1" ht="14.25" spans="1:4">
+      <c r="A31" s="2" t="s">
+        <v>500</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>501</v>
+      </c>
+      <c r="D31" s="10">
         <v>389</v>
       </c>
     </row>
+    <row r="35" s="3" customFormat="1" ht="25.5" spans="1:1">
+      <c r="A35" s="6" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="36" s="3" customFormat="1" ht="25.5"/>
+    <row r="37" s="3" customFormat="1" ht="25.5"/>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A35:XFD37"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555556" footer="0.511805555555556"/>
   <headerFooter/>
 </worksheet>
@@ -5715,8 +5902,8 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr/>
-  <dimension ref="A1:E25"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="4"/>
+  <dimension ref="A1:XFD25"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="20.75" customWidth="1"/>
     <col min="3" max="3" width="64.875" customWidth="1"/>
@@ -5730,7 +5917,7 @@
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="4" t="s">
         <v>2</v>
       </c>
       <c r="E1" s="1" t="s">
@@ -5739,82 +5926,86 @@
     </row>
     <row r="3" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A3" s="2" t="s">
-        <v>491</v>
+        <v>502</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>492</v>
+        <v>503</v>
       </c>
     </row>
     <row r="4" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A4" s="2" t="s">
-        <v>493</v>
+        <v>504</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>494</v>
+        <v>505</v>
       </c>
     </row>
     <row r="5" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A5" s="2" t="s">
-        <v>495</v>
+        <v>506</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>496</v>
+        <v>507</v>
       </c>
     </row>
     <row r="6" s="2" customFormat="1" ht="96" customHeight="1" spans="1:3">
       <c r="A6" s="2" t="s">
-        <v>497</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>498</v>
+        <v>508</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>509</v>
       </c>
     </row>
     <row r="7" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A7" s="2" t="s">
-        <v>499</v>
+        <v>510</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>500</v>
+        <v>511</v>
       </c>
     </row>
     <row r="8" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A8" s="2" t="s">
-        <v>501</v>
+        <v>512</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>502</v>
+        <v>513</v>
       </c>
     </row>
     <row r="9" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A9" s="2" t="s">
-        <v>503</v>
+        <v>514</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>504</v>
+        <v>515</v>
       </c>
     </row>
     <row r="10" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A10" s="2" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>506</v>
+        <v>517</v>
       </c>
     </row>
     <row r="11" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A11" s="2" t="s">
-        <v>507</v>
+        <v>518</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>508</v>
+        <v>519</v>
       </c>
     </row>
     <row r="12" s="2" customFormat="1" ht="14.25"/>
     <row r="13" s="2" customFormat="1" ht="14.25"/>
     <row r="14" s="2" customFormat="1" ht="14.25"/>
-    <row r="15" s="2" customFormat="1" ht="14.25"/>
-    <row r="16" s="2" customFormat="1" ht="14.25"/>
-    <row r="17" s="2" customFormat="1" ht="14.25"/>
+    <row r="15" s="3" customFormat="1" ht="25.5" spans="1:1">
+      <c r="A15" s="6" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="16" s="3" customFormat="1" ht="25.5"/>
+    <row r="17" s="3" customFormat="1" ht="25.5"/>
     <row r="18" s="2" customFormat="1" ht="14.25"/>
     <row r="19" s="2" customFormat="1" ht="14.25"/>
     <row r="20" s="2" customFormat="1" ht="14.25"/>
@@ -5824,6 +6015,9 @@
     <row r="24" s="2" customFormat="1" ht="14.25"/>
     <row r="25" s="2" customFormat="1" ht="14.25"/>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A15:XFD17"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555556" footer="0.511805555555556"/>
   <headerFooter/>
 </worksheet>
@@ -5832,8 +6026,8 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr/>
-  <dimension ref="A1:E84"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="4"/>
+  <dimension ref="A1:XFD84"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="17.125" customWidth="1"/>
     <col min="3" max="3" width="68.25" customWidth="1"/>
@@ -5848,7 +6042,7 @@
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="4" t="s">
         <v>2</v>
       </c>
       <c r="E1" s="1" t="s">
@@ -5857,507 +6051,507 @@
     </row>
     <row r="3" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A3" s="2" t="s">
-        <v>509</v>
+        <v>520</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>510</v>
+        <v>521</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>511</v>
+        <v>522</v>
       </c>
     </row>
     <row r="4" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A4" s="2" t="s">
-        <v>512</v>
+        <v>523</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>513</v>
+        <v>524</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>514</v>
+        <v>525</v>
       </c>
     </row>
     <row r="5" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A5" s="2" t="s">
-        <v>515</v>
+        <v>526</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>516</v>
+        <v>527</v>
       </c>
     </row>
     <row r="6" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A6" s="2" t="s">
-        <v>517</v>
+        <v>528</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>518</v>
+        <v>529</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>519</v>
+        <v>530</v>
       </c>
     </row>
     <row r="7" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A7" s="2" t="s">
-        <v>520</v>
+        <v>531</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>521</v>
+        <v>532</v>
       </c>
     </row>
     <row r="8" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A8" s="2" t="s">
-        <v>522</v>
+        <v>533</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>523</v>
+        <v>534</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>524</v>
+        <v>535</v>
       </c>
     </row>
     <row r="9" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A9" s="2" t="s">
-        <v>525</v>
+        <v>536</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>526</v>
+        <v>537</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>527</v>
+        <v>538</v>
       </c>
     </row>
     <row r="10" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A10" s="2" t="s">
-        <v>528</v>
+        <v>539</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>529</v>
+        <v>540</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>530</v>
+        <v>541</v>
       </c>
     </row>
     <row r="11" s="2" customFormat="1" ht="14.25"/>
     <row r="12" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A12" s="2" t="s">
-        <v>531</v>
+        <v>542</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>532</v>
+        <v>543</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>533</v>
+        <v>544</v>
       </c>
     </row>
     <row r="13" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A13" s="2" t="s">
-        <v>534</v>
+        <v>545</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>535</v>
+        <v>546</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>536</v>
+        <v>547</v>
       </c>
     </row>
     <row r="14" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A14" s="2" t="s">
-        <v>537</v>
+        <v>548</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>538</v>
+        <v>549</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>539</v>
+        <v>550</v>
       </c>
     </row>
     <row r="15" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A15" s="2" t="s">
-        <v>540</v>
+        <v>551</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>541</v>
+        <v>552</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>540</v>
+        <v>551</v>
       </c>
     </row>
     <row r="16" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A16" s="2" t="s">
-        <v>542</v>
+        <v>553</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>543</v>
+        <v>554</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>544</v>
+        <v>555</v>
       </c>
     </row>
     <row r="17" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A17" s="2" t="s">
-        <v>545</v>
+        <v>556</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>546</v>
+        <v>557</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>547</v>
+        <v>558</v>
       </c>
     </row>
     <row r="18" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A18" s="2" t="s">
-        <v>548</v>
+        <v>559</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>549</v>
+        <v>560</v>
       </c>
     </row>
     <row r="19" s="2" customFormat="1" ht="14.25"/>
     <row r="20" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A20" s="2" t="s">
-        <v>550</v>
+        <v>561</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>551</v>
+        <v>562</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>552</v>
+        <v>563</v>
       </c>
     </row>
     <row r="21" s="2" customFormat="1" ht="14.25"/>
     <row r="22" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A22" s="2" t="s">
-        <v>553</v>
+        <v>564</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>554</v>
+        <v>565</v>
       </c>
     </row>
     <row r="23" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A23" s="2" t="s">
-        <v>555</v>
+        <v>566</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>554</v>
+        <v>565</v>
       </c>
     </row>
     <row r="24" s="2" customFormat="1" ht="14.25"/>
     <row r="25" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A25" s="2" t="s">
-        <v>556</v>
+        <v>567</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>557</v>
+        <v>568</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>558</v>
+        <v>569</v>
       </c>
     </row>
     <row r="26" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A26" s="2" t="s">
-        <v>559</v>
+        <v>570</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>560</v>
+        <v>571</v>
       </c>
     </row>
     <row r="27" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A27" s="2" t="s">
-        <v>561</v>
+        <v>572</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>562</v>
+        <v>573</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>563</v>
+        <v>574</v>
       </c>
     </row>
     <row r="28" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A28" s="2" t="s">
-        <v>564</v>
+        <v>575</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>565</v>
+        <v>576</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>566</v>
+        <v>577</v>
       </c>
     </row>
     <row r="29" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A29" s="2" t="s">
-        <v>567</v>
+        <v>578</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>568</v>
+        <v>579</v>
       </c>
     </row>
     <row r="30" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A30" s="2" t="s">
-        <v>569</v>
+        <v>580</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>570</v>
+        <v>581</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>571</v>
+        <v>582</v>
       </c>
     </row>
     <row r="31" s="2" customFormat="1" ht="14.25"/>
     <row r="32" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A32" s="2" t="s">
-        <v>572</v>
+        <v>583</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>573</v>
-      </c>
-      <c r="E32" s="2" t="s">
-        <v>574</v>
+        <v>584</v>
+      </c>
+      <c r="E32" s="7" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="33" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A33" s="2" t="s">
-        <v>575</v>
+        <v>586</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>576</v>
+        <v>587</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>577</v>
+        <v>588</v>
       </c>
     </row>
     <row r="34" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A34" s="2" t="s">
-        <v>578</v>
+        <v>589</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>579</v>
+        <v>590</v>
       </c>
     </row>
     <row r="35" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A35" s="2" t="s">
-        <v>580</v>
+        <v>591</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>581</v>
-      </c>
-      <c r="E35" s="2" t="s">
-        <v>582</v>
+        <v>592</v>
+      </c>
+      <c r="E35" s="7" t="s">
+        <v>593</v>
       </c>
     </row>
     <row r="36" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A36" s="2" t="s">
-        <v>583</v>
+        <v>594</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>584</v>
-      </c>
-      <c r="E36" s="2" t="s">
-        <v>585</v>
+        <v>595</v>
+      </c>
+      <c r="E36" s="7" t="s">
+        <v>596</v>
       </c>
     </row>
     <row r="37" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A37" s="2" t="s">
-        <v>586</v>
+        <v>597</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>587</v>
-      </c>
-      <c r="E37" s="2" t="s">
-        <v>588</v>
+        <v>598</v>
+      </c>
+      <c r="E37" s="7" t="s">
+        <v>599</v>
       </c>
     </row>
     <row r="38" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A38" s="2" t="s">
-        <v>589</v>
-      </c>
-      <c r="C38" s="2" t="s">
-        <v>590</v>
+        <v>600</v>
+      </c>
+      <c r="C38" s="7" t="s">
+        <v>601</v>
       </c>
     </row>
     <row r="39" s="2" customFormat="1" ht="14.25"/>
     <row r="40" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A40" s="2" t="s">
-        <v>591</v>
+        <v>602</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>592</v>
+        <v>603</v>
       </c>
     </row>
     <row r="41" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A41" s="2" t="s">
-        <v>593</v>
+        <v>604</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>594</v>
+        <v>605</v>
       </c>
     </row>
     <row r="42" s="2" customFormat="1" ht="57" spans="1:3">
       <c r="A42" s="2" t="s">
-        <v>595</v>
-      </c>
-      <c r="C42" s="4" t="s">
-        <v>596</v>
+        <v>606</v>
+      </c>
+      <c r="C42" s="5" t="s">
+        <v>607</v>
       </c>
     </row>
     <row r="43" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A43" s="2" t="s">
-        <v>597</v>
+        <v>608</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>598</v>
+        <v>609</v>
       </c>
     </row>
     <row r="44" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A44" s="2" t="s">
-        <v>599</v>
+        <v>610</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>600</v>
+        <v>611</v>
       </c>
     </row>
     <row r="45" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A45" s="2" t="s">
-        <v>601</v>
+        <v>612</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>602</v>
+        <v>613</v>
       </c>
     </row>
     <row r="46" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A46" s="2" t="s">
-        <v>603</v>
+        <v>614</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>604</v>
+        <v>615</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>605</v>
+        <v>616</v>
       </c>
     </row>
     <row r="47" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A47" s="2" t="s">
-        <v>606</v>
+        <v>617</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>607</v>
+        <v>618</v>
       </c>
     </row>
     <row r="48" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A48" s="2" t="s">
-        <v>608</v>
+        <v>619</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>609</v>
+        <v>620</v>
       </c>
     </row>
     <row r="49" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A49" s="2" t="s">
-        <v>610</v>
+        <v>621</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>611</v>
+        <v>622</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>612</v>
+        <v>623</v>
       </c>
     </row>
     <row r="50" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A50" s="2" t="s">
-        <v>613</v>
+        <v>624</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>614</v>
+        <v>625</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>615</v>
+        <v>626</v>
       </c>
     </row>
     <row r="51" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A51" s="2" t="s">
-        <v>616</v>
+        <v>627</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>617</v>
+        <v>628</v>
       </c>
     </row>
     <row r="52" s="2" customFormat="1" ht="28.5" spans="1:3">
       <c r="A52" s="2" t="s">
-        <v>618</v>
-      </c>
-      <c r="C52" s="4" t="s">
-        <v>619</v>
+        <v>629</v>
+      </c>
+      <c r="C52" s="5" t="s">
+        <v>630</v>
       </c>
     </row>
     <row r="53" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A53" s="2" t="s">
-        <v>620</v>
+        <v>631</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>621</v>
+        <v>632</v>
       </c>
     </row>
     <row r="54" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A54" s="2" t="s">
-        <v>622</v>
+        <v>633</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>623</v>
+        <v>634</v>
       </c>
     </row>
     <row r="55" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A55" s="2" t="s">
-        <v>624</v>
+        <v>635</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>625</v>
+        <v>636</v>
       </c>
     </row>
     <row r="56" s="2" customFormat="1" ht="14.25"/>
     <row r="57" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A57" s="2" t="s">
-        <v>626</v>
+        <v>637</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>627</v>
+        <v>638</v>
       </c>
     </row>
     <row r="58" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A58" s="2" t="s">
-        <v>628</v>
+        <v>639</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>629</v>
+        <v>640</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>630</v>
+        <v>641</v>
       </c>
     </row>
     <row r="59" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A59" s="2" t="s">
-        <v>631</v>
+        <v>642</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>632</v>
+        <v>643</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>633</v>
+        <v>644</v>
       </c>
     </row>
     <row r="60" s="2" customFormat="1" ht="14.25"/>
     <row r="61" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A61" s="2" t="s">
-        <v>634</v>
+        <v>645</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>635</v>
+        <v>646</v>
       </c>
     </row>
     <row r="62" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A62" s="2" t="s">
-        <v>636</v>
+        <v>647</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>637</v>
+        <v>648</v>
       </c>
     </row>
     <row r="63" s="2" customFormat="1" ht="14.25" spans="1:3">
@@ -6365,7 +6559,7 @@
         <v>125</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>638</v>
+        <v>649</v>
       </c>
     </row>
     <row r="64" s="2" customFormat="1" ht="14.25" spans="1:3">
@@ -6373,120 +6567,127 @@
         <v>127</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>639</v>
+        <v>650</v>
       </c>
     </row>
     <row r="65" s="2" customFormat="1" ht="14.25"/>
     <row r="66" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A66" s="2" t="s">
-        <v>640</v>
+        <v>651</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>641</v>
+        <v>652</v>
       </c>
       <c r="E66" s="2" t="s">
-        <v>642</v>
+        <v>653</v>
       </c>
     </row>
     <row r="67" s="2" customFormat="1" ht="14.25" spans="1:5">
       <c r="A67" s="2" t="s">
-        <v>643</v>
+        <v>654</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>644</v>
+        <v>655</v>
       </c>
       <c r="E67" s="2" t="s">
-        <v>645</v>
+        <v>656</v>
       </c>
     </row>
     <row r="68" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A68" s="2" t="s">
-        <v>646</v>
+        <v>657</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>647</v>
+        <v>658</v>
       </c>
     </row>
     <row r="69" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A69" s="2" t="s">
-        <v>648</v>
+        <v>659</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>649</v>
+        <v>660</v>
       </c>
     </row>
     <row r="70" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A70" s="2" t="s">
-        <v>650</v>
+        <v>661</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>651</v>
+        <v>662</v>
       </c>
     </row>
     <row r="71" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A71" s="2" t="s">
-        <v>652</v>
+        <v>663</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>653</v>
+        <v>664</v>
       </c>
     </row>
     <row r="72" s="2" customFormat="1" ht="14.25"/>
     <row r="73" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A73" s="2" t="s">
-        <v>654</v>
+        <v>665</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>655</v>
+        <v>666</v>
       </c>
     </row>
     <row r="74" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A74" s="2" t="s">
-        <v>656</v>
+        <v>667</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>657</v>
+        <v>668</v>
       </c>
     </row>
     <row r="75" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A75" s="2" t="s">
-        <v>658</v>
+        <v>669</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>659</v>
+        <v>670</v>
       </c>
     </row>
     <row r="76" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A76" s="2" t="s">
-        <v>660</v>
+        <v>671</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>661</v>
+        <v>672</v>
       </c>
     </row>
     <row r="77" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A77" s="2" t="s">
-        <v>662</v>
+        <v>673</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>663</v>
+        <v>674</v>
       </c>
     </row>
     <row r="78" s="2" customFormat="1" ht="14.25" spans="1:3">
       <c r="A78" s="2" t="s">
-        <v>664</v>
+        <v>675</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>665</v>
+        <v>676</v>
       </c>
     </row>
     <row r="79" s="2" customFormat="1" ht="14.25"/>
     <row r="80" s="2" customFormat="1" ht="14.25"/>
     <row r="81" s="2" customFormat="1" ht="14.25"/>
-    <row r="82" s="2" customFormat="1" ht="14.25"/>
-    <row r="83" s="2" customFormat="1" ht="14.25"/>
-    <row r="84" s="2" customFormat="1" ht="14.25"/>
+    <row r="82" s="3" customFormat="1" ht="25.5" spans="1:1">
+      <c r="A82" s="6" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="83" s="3" customFormat="1" ht="25.5"/>
+    <row r="84" s="3" customFormat="1" ht="25.5"/>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A82:XFD84"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555556" footer="0.511805555555556"/>
   <headerFooter/>
 </worksheet>

</xml_diff>